<commit_message>
Update Arbeitsrapport_ Projekt_Khalil's Gym.xlsx
</commit_message>
<xml_diff>
--- a/Arbeitsrapport_ Projekt_Khalil's Gym.xlsx
+++ b/Arbeitsrapport_ Projekt_Khalil's Gym.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Khalil Hamahmi\OneDrive - sluz\Dokumente\GitHub\IPT_4.1-Projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859197BF-B928-488D-99EF-B5238FA08544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BC0DF1-4C65-40AD-8C19-FC5425E93E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{0E4E67A2-2C85-46AE-B51D-DC0506011435}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>Arbeitsplanung</t>
   </si>
@@ -108,6 +108,12 @@
   </si>
   <si>
     <t>Data Grip mit Docker verbinden</t>
+  </si>
+  <si>
+    <t>Api erstellt und testdaten anzeigen</t>
+  </si>
+  <si>
+    <t>35 Minuten</t>
   </si>
 </sst>
 </file>
@@ -853,10 +859,18 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C13" s="3"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="C13" s="3">
+        <v>45989</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">

</xml_diff>